<commit_message>
Refresh KS_Mapping_Table.xlsx line references after Jack's question-enhancements removal
</commit_message>
<xml_diff>
--- a/KS_Mapping_Table.xlsx
+++ b/KS_Mapping_Table.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:38; Formulate_Response_PD_Broad_to_Narrow.yaml:308; Formulate_Response_PD_Broad_to_Narrow.yaml:444; Formulate_Response_Programme_Development_File_Upload.yaml:117; Formulate_Response_Programme_Development_File_Upload.yaml:420; Formulate_Response_Programme_Development_File_Upload.yaml:459</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:38; Formulate_Response_PD_Broad_to_Narrow.yaml:308; Formulate_Response_PD_Broad_to_Narrow.yaml:444; Formulate_Response_Programme_Development_File_Upload.yaml:111; Formulate_Response_Programme_Development_File_Upload.yaml:402; Formulate_Response_Programme_Development_File_Upload.yaml:439</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:84; Formulate_Response_Programme_Development_File_Upload.yaml:45</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:84; Formulate_Response_Programme_Development_File_Upload.yaml:43</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:121; Formulate_Response_Programme_Development_File_Upload.yaml:81</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:121; Formulate_Response_Programme_Development_File_Upload.yaml:77</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:158; Formulate_Response_Programme_Development_File_Upload.yaml:152</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:158; Formulate_Response_Programme_Development_File_Upload.yaml:144</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:195; Formulate_Response_Programme_Development_File_Upload.yaml:187</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:195; Formulate_Response_Programme_Development_File_Upload.yaml:177</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:232; Formulate_Response_Programme_Development_File_Upload.yaml:222</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:232; Formulate_Response_Programme_Development_File_Upload.yaml:210</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:233; Formulate_Response_Programme_Development_File_Upload.yaml:223</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:233; Formulate_Response_Programme_Development_File_Upload.yaml:211</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:270; Formulate_Response_Programme_Development_File_Upload.yaml:258</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:270; Formulate_Response_Programme_Development_File_Upload.yaml:244</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:374; Formulate_Response_Programme_Development_File_Upload.yaml:354</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:374; Formulate_Response_Programme_Development_File_Upload.yaml:340</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:411; Formulate_Response_Programme_Development_File_Upload.yaml:389</t>
+          <t>Formulate_Response_PD_Broad_to_Narrow.yaml:411; Formulate_Response_Programme_Development_File_Upload.yaml:373</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>Auto-matched - please confirm</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">

</xml_diff>